<commit_message>
RECORD P06 is 1087453, 1097453 off (10505->10509); review and branch list rebuilt on 10509
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968862_Buildings_for_Branch_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968862_Buildings_for_Branch_22Oct2026.xlsx
@@ -1078,86 +1078,82 @@
       <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Building 6m</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>1097453</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1087453</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>1087453</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>P06</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>1426.07</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="M9" s="2" t="n">
+      <c r="M9" t="n">
         <v>353.94</v>
       </c>
-      <c r="N9" s="2" t="n">
-        <v>145.74</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="P9" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="Q9" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>line has asset 1087453 - site number is 1097453</t>
-        </is>
-      </c>
+      <c r="N9" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="O9" t="n">
+        <v>500</v>
+      </c>
+      <c r="P9" t="n">
+        <v>500</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>500</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">

</xml_diff>

<commit_message>
v11.19 LIVE (GN24 is the 60 kVA 1277089, line 17 never came); record: AA and HRP tracked not charged; generators workbook on 14 sets; branch building list
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968862_Buildings_for_Branch_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9968862_Buildings_for_Branch_22Oct2026.xlsx
@@ -561,47 +561,45 @@
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>510.09</v>
+        <v>0</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>145.74</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>500</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>no hire line - add</t>
+          <t>tracked only - paid on the customer's own contract HS 9968926 (Active Air); no charge on 9968862 - right that it has no line</t>
         </is>
       </c>
     </row>
@@ -721,47 +719,45 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no charge</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>510.09</v>
+        <v>0</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>145.74</v>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>500</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>line labelled P36 - relabel HRP</t>
+          <t>tracked only - paid on the customer's own contract HS 9974238 (Hire Republic); no charge on 9968862 - line 93 comes off this contract</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4209,7 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>47 buildings</t>
+          <t>45 buildings charged</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr"/>
@@ -4222,34 +4218,38 @@
       <c r="F50" s="1" t="inlineStr"/>
       <c r="G50" s="1" t="inlineStr"/>
       <c r="H50" s="1" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I50" s="1" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J50" s="1" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K50" s="1" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="L50" s="1" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="M50" s="1" t="n">
-        <v>22881.18</v>
+        <v>21861</v>
       </c>
       <c r="N50" s="1" t="n">
-        <v>6849.78</v>
+        <v>6558.3</v>
       </c>
       <c r="O50" s="1" t="inlineStr"/>
       <c r="P50" s="1" t="n">
-        <v>26200</v>
+        <v>25200</v>
       </c>
       <c r="Q50" s="1" t="n">
-        <v>26200</v>
-      </c>
-      <c r="R50" s="1" t="inlineStr"/>
+        <v>25200</v>
+      </c>
+      <c r="R50" s="1" t="inlineStr">
+        <is>
+          <t>2 tracked only (AA, HRP), not charged on 9968862</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4262,7 +4262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -4303,6 +4303,13 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AA (Active Air) and HRP (Hire Republic) are on site and tracked, but each customer pays for its building on its own contract (HS 9968926, HS 9974238): no hire, labour, steps, transport or demob is charged on 9968862. Line 93 (1189410) comes off this contract.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>